<commit_message>
Updated Excel seeder to include passwords for secure login
</commit_message>
<xml_diff>
--- a/mock_university_database.xlsx
+++ b/mock_university_database.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -437,6 +437,7 @@
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="29" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,6 +466,11 @@
           <t>hire_year</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>password</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -488,6 +494,11 @@
       <c r="E2" t="n">
         <v>2015</v>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Pass123!</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -511,6 +522,11 @@
       <c r="E3" t="n">
         <v>2010</v>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Pass123!</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -534,6 +550,11 @@
       <c r="E4" t="n">
         <v>2005</v>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Pass123!</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -557,6 +578,11 @@
       <c r="E5" t="n">
         <v>2020</v>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Pass123!</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -580,6 +606,11 @@
       <c r="E6" t="n">
         <v>2025</v>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Pass123!</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -603,6 +634,11 @@
       <c r="E7" t="n">
         <v>2018</v>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Pass123!</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -625,6 +661,11 @@
       </c>
       <c r="E8" t="n">
         <v>2021</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Pass123!</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added ValueError exception to handle blank Excel cells
</commit_message>
<xml_diff>
--- a/mock_university_database.xlsx
+++ b/mock_university_database.xlsx
@@ -429,15 +429,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="29" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -463,11 +462,6 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>hire_year</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
           <t>password</t>
         </is>
       </c>
@@ -491,10 +485,7 @@
           <t>Category 2 (Professional)</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>2015</v>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Pass123!</t>
         </is>
@@ -519,10 +510,7 @@
           <t>Category 1 (Management)</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>2010</v>
-      </c>
-      <c r="F3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Pass123!</t>
         </is>
@@ -534,23 +522,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dr. Charlie School</t>
+          <t>Veteran Val</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>HoS</t>
+          <t>Senior Lecturer</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Category 1 (Management)</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>2005</v>
-      </c>
-      <c r="F4" t="inlineStr">
+          <t>Category 4 (PhD Staff)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>Pass123!</t>
         </is>
@@ -562,23 +547,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Veteran Val</t>
+          <t>Newbie Nick</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Senior Lecturer</t>
+          <t>Lecturer</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Category 4 (PhD Staff)</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>2020</v>
-      </c>
-      <c r="F5" t="inlineStr">
+          <t>Category 5 (Other Academic)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>Pass123!</t>
         </is>
@@ -590,7 +572,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Newbie Nick</t>
+          <t>Test Terry</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -598,75 +580,8 @@
           <t>Lecturer</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Category 5 (Other Academic)</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>2025</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Pass123!</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Dr. Dave</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Associate Professor</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Category 4 (PhD Staff)</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>2018</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Pass123!</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Lecturer Larry</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Lecturer</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Category 5 (Other Academic)</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>2021</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Pass123!</t>
-        </is>
-      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -679,11 +594,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
   </cols>
@@ -760,81 +675,7 @@
       <c r="C4" t="n">
         <v>4</v>
       </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>CS301</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Artificial Intelligence</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D5" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>CS302</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Database Systems</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>CS401</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Cloud Computing</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>CS405</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Software Engineering</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>3</v>
-      </c>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
+      <c r="D4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -847,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -903,76 +744,11 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>CS201</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="n">
-        <v>5</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CS301</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="n">
-        <v>6</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CS302</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="n">
-        <v>6</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CS401</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="n">
-        <v>6</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CS405</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="n">
-        <v>7</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CS101</t>
         </is>
       </c>
     </row>
@@ -987,14 +763,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1018,32 +793,22 @@
           <t>proposed_category</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Professor</t>
+          <t>Senior Lecturer</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>Category 4 (PhD Staff)</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Pending HoD</t>
         </is>
       </c>
     </row>
@@ -1063,7 +828,7 @@
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="81" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
   </cols>
@@ -1100,11 +865,11 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>I would like to request an additional practical assistant for the CS301 module.</t>
+          <t>Testing the new robust seeder!</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1114,7 +879,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Developed tabbed HoD Dashboard with promotion approval pipeline
</commit_message>
<xml_diff>
--- a/mock_university_database.xlsx
+++ b/mock_university_database.xlsx
@@ -429,14 +429,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="29" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -462,6 +463,11 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>hire_year</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>password</t>
         </is>
       </c>
@@ -485,7 +491,10 @@
           <t>Category 2 (Professional)</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" t="n">
+        <v>2015</v>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>Pass123!</t>
         </is>
@@ -510,7 +519,10 @@
           <t>Category 1 (Management)</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" t="n">
+        <v>2010</v>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>Pass123!</t>
         </is>
@@ -522,20 +534,23 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Veteran Val</t>
+          <t>Dr. Charlie School</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Senior Lecturer</t>
+          <t>HoS</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Category 4 (PhD Staff)</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+          <t>Category 1 (Management)</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>2005</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Pass123!</t>
         </is>
@@ -547,20 +562,23 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Newbie Nick</t>
+          <t>Veteran Val</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Lecturer</t>
+          <t>Senior Lecturer</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Category 5 (Other Academic)</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+          <t>Category 4 (PhD Staff)</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>2020</v>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>Pass123!</t>
         </is>
@@ -572,7 +590,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Test Terry</t>
+          <t>Newbie Nick</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -580,8 +598,75 @@
           <t>Lecturer</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Category 5 (Other Academic)</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Pass123!</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Dr. Dave</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Category 4 (PhD Staff)</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2018</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Pass123!</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Lecturer Larry</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Category 5 (Other Academic)</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>2021</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Pass123!</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -594,11 +679,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
   </cols>
@@ -675,7 +760,81 @@
       <c r="C4" t="n">
         <v>4</v>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CS301</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CS302</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Database Systems</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CS401</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Cloud Computing</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CS405</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Software Engineering</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -688,7 +847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -744,11 +903,76 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CS201</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
         <v>5</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CS201</t>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CS301</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CS302</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CS401</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CS405</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>7</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CS101</t>
         </is>
       </c>
     </row>
@@ -763,13 +987,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -793,22 +1018,32 @@
           <t>proposed_category</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Senior Lecturer</t>
+          <t>Professor</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>Category 4 (PhD Staff)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Pending HoD</t>
         </is>
       </c>
     </row>
@@ -828,7 +1063,7 @@
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="81" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
   </cols>
@@ -865,11 +1100,11 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Testing the new robust seeder!</t>
+          <t>I would like to request an additional practical assistant for the CS301 module.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -879,7 +1114,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-22</t>
         </is>
       </c>
     </row>

</xml_diff>